<commit_message>
Complete MNIST digit recognition model and evaluation
</commit_message>
<xml_diff>
--- a/architecture_results.xlsx
+++ b/architecture_results.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Sparsh Python Programming folder\handwritten digits recognition\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C208EDC-E300-4895-9617-9AF327F4477F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55E30EFF-E18F-4CEF-81A7-A0DB11BDB006}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Sr No</t>
   </si>
@@ -46,39 +46,55 @@
     <t>196 → 64</t>
   </si>
   <si>
+    <t>196 → 32</t>
+  </si>
+  <si>
     <t>128 → 98</t>
   </si>
   <si>
     <t>128 → 64</t>
   </si>
   <si>
-    <t>Key:</t>
-  </si>
-  <si>
-    <t>Meaning</t>
-  </si>
-  <si>
-    <t>Bold and Bigger Font</t>
-  </si>
-  <si>
-    <t>Best Accuracy or Loss</t>
-  </si>
-  <si>
-    <t>Selected Hyperparameter</t>
+    <t>128 → 32</t>
+  </si>
+  <si>
+    <t>98 → 98</t>
+  </si>
+  <si>
+    <t>98 → 64</t>
+  </si>
+  <si>
+    <t>98 → 32</t>
+  </si>
+  <si>
+    <t>Key</t>
+  </si>
+  <si>
+    <t>Bold and bigger font</t>
+  </si>
+  <si>
+    <t>Best observation for that feature</t>
+  </si>
+  <si>
+    <t>Selected Architecture</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="167" formatCode="0.0000"/>
-    <numFmt numFmtId="171" formatCode="0.0"/>
-  </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -92,7 +108,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -101,12 +117,23 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -114,32 +141,55 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </left>
+      <right style="thin">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </right>
+      <top style="thin">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="171" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="167" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Calculation" xfId="1" builtinId="22"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
-    <dxf>
-      <numFmt numFmtId="167" formatCode="0.0000"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="0.0000"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -153,28 +203,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{19AB7DA2-C302-41B6-B90B-5BAB5D136EB6}" name="Table1" displayName="Table1" ref="A1:F5" totalsRowShown="0">
-  <autoFilter ref="A1:F5" xr:uid="{19AB7DA2-C302-41B6-B90B-5BAB5D136EB6}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{CF4C25A7-C0F1-4188-B61B-BA24253D379B}" name="Table2" displayName="Table2" ref="A1:F10" totalsRowShown="0">
+  <autoFilter ref="A1:F10" xr:uid="{CF4C25A7-C0F1-4188-B61B-BA24253D379B}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{D05F003A-B981-4A4E-BE0A-B402F7963A70}" name="Sr No"/>
-    <tableColumn id="2" xr3:uid="{C0C437DD-4045-418C-8359-76A3E38C2C93}" name="Architecture"/>
-    <tableColumn id="3" xr3:uid="{137DD3A4-502B-4153-BA2A-BE7E0690CD56}" name="Validation Accuracy" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{C6E8B5E3-8350-4F10-8CA6-4FB3CE34DB2E}" name="Validation Loss" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{6A4521DD-1556-4A03-9A7D-DA28CDE3F15A}" name="Training Loss" dataDxfId="0"/>
-    <tableColumn id="6" xr3:uid="{20C136D5-890B-4980-8232-C54FBE6CCC53}" name="Epochs"/>
+    <tableColumn id="1" xr3:uid="{43851901-5AB8-4B59-8FD2-76450D16C88A}" name="Sr No"/>
+    <tableColumn id="2" xr3:uid="{D45FAA67-D564-4680-AD8F-E548D7BDE7A8}" name="Architecture"/>
+    <tableColumn id="3" xr3:uid="{752D6797-70A7-4C38-A484-211840FDCD49}" name="Validation Accuracy"/>
+    <tableColumn id="4" xr3:uid="{83952703-67ED-4ABE-94F8-B3247F11CFA2}" name="Validation Loss"/>
+    <tableColumn id="5" xr3:uid="{A1F062C2-EC9B-4E0D-BE1F-0DDD1FD02A5A}" name="Training Loss"/>
+    <tableColumn id="6" xr3:uid="{7855A67D-1D68-4806-A46A-BF9230AC1389}" name="Epochs"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{455B3B9E-2D51-4806-84E0-9DDD5A8E0FAC}" name="Table3" displayName="Table3" ref="H3:I5" totalsRowShown="0">
-  <autoFilter ref="H3:I5" xr:uid="{455B3B9E-2D51-4806-84E0-9DDD5A8E0FAC}"/>
-  <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{57C0F3C9-3436-467F-99C7-932ACC7BDC02}" name="Key:"/>
-    <tableColumn id="2" xr3:uid="{B81E2D86-27B9-41B3-BEFE-9B54AC5EF7FA}" name="Meaning"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -461,17 +500,52 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="525" row="1">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{F5F77FEB-9A0E-44F2-A369-4366362CE2AA}">
+  <we:reference id="wa200007447" version="1.1.6.7" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="wa200007447" version="1.1.6.7" store="wa200007447" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties/>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+  <we:extLst>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{D87F86FE-615C-45B5-9D79-34F1136793EB}">
+      <we:containsCustomFunctions/>
+    </a:ext>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{7C84B067-C214-45C3-A712-C9D94CD141B2}">
+      <we:customFunctionIdList>
+        <we:customFunctionIds>_xldudf_BOARDFLARE_EXEC</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_BF_OUTPUT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_BF_FUNCTION</we:customFunctionIds>
+      </we:customFunctionIdList>
+    </a:ext>
+  </we:extLst>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I5"/>
+  <sheetPr>
+    <tabColor theme="4"/>
+  </sheetPr>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="13.1796875" customWidth="1"/>
     <col min="3" max="3" width="19.1796875" customWidth="1"/>
     <col min="4" max="4" width="15.36328125" customWidth="1"/>
     <col min="5" max="5" width="13.54296875" customWidth="1"/>
-    <col min="8" max="8" width="18.08984375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22.26953125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="28.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
@@ -494,107 +568,204 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="4">
-        <v>97.891666666666666</v>
-      </c>
-      <c r="D2" s="5">
-        <v>7.6238805614411834E-2</v>
-      </c>
-      <c r="E2" s="5">
-        <v>1.455098539113533E-2</v>
-      </c>
-      <c r="F2" s="3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="C2">
+        <v>97.93</v>
+      </c>
+      <c r="D2">
+        <v>7.5300000000000006E-2</v>
+      </c>
+      <c r="E2">
+        <v>1.4E-2</v>
+      </c>
+      <c r="F2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="2">
-        <v>97.766666666666666</v>
-      </c>
-      <c r="D3" s="1">
-        <v>8.0805195684234304E-2</v>
+      <c r="C3">
+        <v>97.83</v>
+      </c>
+      <c r="D3">
+        <v>8.0500000000000002E-2</v>
       </c>
       <c r="E3" s="1">
-        <v>1.5842869279440491E-2</v>
+        <v>1.37E-2</v>
       </c>
       <c r="F3">
         <v>10</v>
       </c>
-      <c r="H3" t="s">
-        <v>10</v>
-      </c>
-      <c r="I3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4">
+    </row>
+    <row r="4" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="2">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="2">
-        <v>97.783333333333331</v>
-      </c>
-      <c r="D4" s="1">
-        <v>7.982203041668981E-2</v>
-      </c>
-      <c r="E4" s="1">
-        <v>2.0872650975594299E-2</v>
-      </c>
-      <c r="F4">
-        <v>10</v>
-      </c>
-      <c r="H4" t="s">
-        <v>12</v>
-      </c>
-      <c r="I4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="C4" s="3">
+        <v>97.96</v>
+      </c>
+      <c r="D4" s="3">
+        <v>7.2900000000000006E-2</v>
+      </c>
+      <c r="E4" s="2">
+        <v>1.7299999999999999E-2</v>
+      </c>
+      <c r="F4" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="2">
-        <v>97.50833333333334</v>
-      </c>
-      <c r="D5" s="1">
-        <v>8.4055603030448164E-2</v>
-      </c>
-      <c r="E5" s="1">
-        <v>2.3717720649515588E-2</v>
+      <c r="C5">
+        <v>97.65</v>
+      </c>
+      <c r="D5">
+        <v>7.7299999999999994E-2</v>
+      </c>
+      <c r="E5">
+        <v>2.1399999999999999E-2</v>
       </c>
       <c r="F5">
         <v>10</v>
       </c>
-      <c r="H5" s="3"/>
-      <c r="I5" t="s">
+      <c r="H5" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="I5" s="4"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6">
+        <v>97.67</v>
+      </c>
+      <c r="D6">
+        <v>7.7799999999999994E-2</v>
+      </c>
+      <c r="E6">
+        <v>2.24E-2</v>
+      </c>
+      <c r="F6">
+        <v>10</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7">
+        <v>97.52</v>
+      </c>
+      <c r="D7">
+        <v>8.3099999999999993E-2</v>
+      </c>
+      <c r="E7">
+        <v>2.64E-2</v>
+      </c>
+      <c r="F7">
+        <v>10</v>
+      </c>
+      <c r="H7" s="5"/>
+      <c r="I7" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8">
+        <v>97.33</v>
+      </c>
+      <c r="D8">
+        <v>0.09</v>
+      </c>
+      <c r="E8">
+        <v>2.9000000000000001E-2</v>
+      </c>
+      <c r="F8">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9">
+        <v>97.6</v>
+      </c>
+      <c r="D9">
+        <v>8.1900000000000001E-2</v>
+      </c>
+      <c r="E9">
+        <v>2.81E-2</v>
+      </c>
+      <c r="F9">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
         <v>14</v>
+      </c>
+      <c r="C10">
+        <v>97.25</v>
+      </c>
+      <c r="D10">
+        <v>8.72E-2</v>
+      </c>
+      <c r="E10">
+        <v>3.6200000000000003E-2</v>
+      </c>
+      <c r="F10">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="2">
+  <tableParts count="1">
     <tablePart r:id="rId1"/>
-    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>